<commit_message>
feat: add raw UMKM survey data and processed spatial files for RW1 analysis
</commit_message>
<xml_diff>
--- a/01_data_mentah/survei_lapangan/data_umkm.xlsx
+++ b/01_data_mentah/survei_lapangan/data_umkm.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace\PetaSebaranUMKM\01_data_mentah\survei_lapangan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DA35DF5-8E62-438F-8188-AF88568DEF36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E99587B2-C45D-4B21-92CC-012EF0FD826A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{61E2F757-5A6D-41CA-B251-E79C00540424}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
   <si>
     <t>id_umkm</t>
   </si>
@@ -126,19 +126,28 @@
     <t>Otak-otak Mak Ucu</t>
   </si>
   <si>
-    <t>0.81462</t>
-  </si>
-  <si>
     <t>Otak-otak Buk Iza</t>
   </si>
   <si>
     <t>Otak-otak Mak Oteh</t>
   </si>
   <si>
-    <t>0.81326</t>
-  </si>
-  <si>
     <t>0.81369</t>
+  </si>
+  <si>
+    <t>foto</t>
+  </si>
+  <si>
+    <t>Cafe Tanjung Lili</t>
+  </si>
+  <si>
+    <t>0.8100192059244234</t>
+  </si>
+  <si>
+    <t>0.814642</t>
+  </si>
+  <si>
+    <t>0.813404</t>
   </si>
 </sst>
 </file>
@@ -498,17 +507,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6378408B-1217-4AC6-A774-844BD89DD224}">
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -516,209 +526,318 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
       <c r="B2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="1">
+      <c r="E2" s="1">
         <v>104595541</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
       <c r="B3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="1">
+      <c r="E3" s="1">
         <v>104595198</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
       <c r="B4" t="s">
         <v>10</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="1">
+      <c r="E4" s="1">
         <v>104595874</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>4</v>
+      </c>
       <c r="B5" t="s">
         <v>11</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="1">
+      <c r="E5" s="1">
         <v>104595188</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>5</v>
+      </c>
       <c r="B6" t="s">
         <v>12</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="1">
+      <c r="E6" s="1">
         <v>104595165</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>6</v>
+      </c>
       <c r="B7" t="s">
         <v>13</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="1">
+      <c r="E7" s="1">
         <v>104595025</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>7</v>
+      </c>
       <c r="B8" t="s">
         <v>14</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="1">
+      <c r="E8" s="1">
         <v>104593897</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>8</v>
+      </c>
       <c r="B9" t="s">
         <v>15</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="1">
+      <c r="E9" s="1">
         <v>104594038</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>9</v>
+      </c>
       <c r="B10" t="s">
         <v>16</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>21</v>
       </c>
-      <c r="D10" s="1">
+      <c r="E10" s="1">
         <v>104594600</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F10">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>10</v>
+      </c>
       <c r="B11" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="2"/>
+      <c r="D11" t="s">
         <v>22</v>
       </c>
-      <c r="D11" s="1">
+      <c r="E11" s="1">
         <v>104593743</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F11">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>11</v>
+      </c>
       <c r="B12" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="2"/>
+      <c r="D12" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="1">
+      <c r="E12" s="1">
         <v>104593709</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F12">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>12</v>
+      </c>
       <c r="B13" t="s">
         <v>27</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>28</v>
       </c>
-      <c r="D13" s="1">
+      <c r="E13" s="1">
         <v>104593421</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F13">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>13</v>
+      </c>
       <c r="B14" t="s">
         <v>29</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
+        <v>36</v>
+      </c>
+      <c r="E14" s="1">
+        <v>104593841</v>
+      </c>
+      <c r="F14">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="1">
-        <v>10459383</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B15" t="s">
+      <c r="D15" t="s">
+        <v>37</v>
+      </c>
+      <c r="E15" s="1">
+        <v>104593850</v>
+      </c>
+      <c r="F15">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
         <v>31</v>
       </c>
-      <c r="C15" t="s">
-        <v>33</v>
-      </c>
-      <c r="D15" s="1">
-        <v>10459385</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B16" t="s">
+      <c r="D16" t="s">
         <v>32</v>
       </c>
-      <c r="C16" t="s">
+      <c r="E16" s="1">
+        <v>10459394</v>
+      </c>
+      <c r="F16">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
         <v>34</v>
       </c>
-      <c r="D16" s="1">
-        <v>10459394</v>
-      </c>
-    </row>
-    <row r="17" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D17" s="1"/>
-    </row>
-    <row r="18" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D18" s="1"/>
-    </row>
-    <row r="19" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D19" s="1"/>
-    </row>
-    <row r="20" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D20" s="1"/>
-    </row>
-    <row r="21" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D21" s="1"/>
-    </row>
-    <row r="22" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D22" s="1"/>
-    </row>
-    <row r="23" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D23" s="1"/>
-    </row>
-    <row r="24" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D24" s="1"/>
-    </row>
-    <row r="25" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D25" s="1"/>
-    </row>
-    <row r="26" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D26" s="1"/>
+      <c r="D17" t="s">
+        <v>35</v>
+      </c>
+      <c r="E17" s="1">
+        <v>1.04592847578478E+16</v>
+      </c>
+      <c r="F17">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E18" s="1"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E19" s="1"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E20" s="1"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E21" s="1"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E22" s="1"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E23" s="1"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E24" s="1"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E25" s="1"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E26" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: import UMKM field survey data, coordinate files, and processed geographical datasets
</commit_message>
<xml_diff>
--- a/01_data_mentah/survei_lapangan/data_umkm.xlsx
+++ b/01_data_mentah/survei_lapangan/data_umkm.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace\PetaSebaranUMKM\01_data_mentah\survei_lapangan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E99587B2-C45D-4B21-92CC-012EF0FD826A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD75AF07-5E61-47B1-AB42-B6B9ED1860D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{61E2F757-5A6D-41CA-B251-E79C00540424}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
   <si>
     <t>id_umkm</t>
   </si>
@@ -132,9 +132,6 @@
     <t>Otak-otak Mak Oteh</t>
   </si>
   <si>
-    <t>0.81369</t>
-  </si>
-  <si>
     <t>foto</t>
   </si>
   <si>
@@ -148,6 +145,15 @@
   </si>
   <si>
     <t>0.813404</t>
+  </si>
+  <si>
+    <t>Otak-otak Buk Yana</t>
+  </si>
+  <si>
+    <t>0.813468</t>
+  </si>
+  <si>
+    <t>0.813698046917283</t>
   </si>
 </sst>
 </file>
@@ -526,7 +532,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D1" t="s">
         <v>2</v>
@@ -752,7 +758,7 @@
         <v>29</v>
       </c>
       <c r="D14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E14" s="1">
         <v>104593841</v>
@@ -769,7 +775,7 @@
         <v>30</v>
       </c>
       <c r="D15" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E15" s="1">
         <v>104593850</v>
@@ -786,10 +792,10 @@
         <v>31</v>
       </c>
       <c r="D16" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="E16" s="1">
-        <v>10459394</v>
+        <v>1.04593886460754E+16</v>
       </c>
       <c r="F16">
         <v>15</v>
@@ -800,10 +806,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
+        <v>33</v>
+      </c>
+      <c r="D17" t="s">
         <v>34</v>
-      </c>
-      <c r="D17" t="s">
-        <v>35</v>
       </c>
       <c r="E17" s="1">
         <v>1.04592847578478E+16</v>
@@ -813,7 +819,21 @@
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E18" s="1"/>
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>37</v>
+      </c>
+      <c r="D18" t="s">
+        <v>38</v>
+      </c>
+      <c r="E18" s="1">
+        <v>104593860</v>
+      </c>
+      <c r="F18">
+        <v>17</v>
+      </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="E19" s="1"/>

</xml_diff>